<commit_message>
New manuscript: combo ch1 and ch2
</commit_message>
<xml_diff>
--- a/Chapter1/Tables/Encapsulated_Apatite.xlsx
+++ b/Chapter1/Tables/Encapsulated_Apatite.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\Dissertation\Chapter1\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\DissertationBJT\Chapter1\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE93CA35-73B3-45AE-BE62-9FBDD8AAB4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C7E12AA-B56D-4656-B9D1-C633CEDBA572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{520F5338-B44B-487F-B878-CEA55A98C4B7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{520F5338-B44B-487F-B878-CEA55A98C4B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data and Corrections" sheetId="6" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="142">
   <si>
     <t>Name</t>
   </si>
@@ -588,6 +588,9 @@
       </rPr>
       <t xml:space="preserve"> Corrected</t>
     </r>
+  </si>
+  <si>
+    <t>C_gas/Cap</t>
   </si>
 </sst>
 </file>
@@ -1220,7 +1223,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1305,6 +1308,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4701,13 +4705,10 @@
       <sheetName val="STDs"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0">
+      <sheetData sheetId="0" refreshError="1">
         <row r="9">
           <cell r="AG9">
             <v>4.9585314106207479E-2</v>
-          </cell>
-          <cell r="AH9">
-            <v>0.23714864603814678</v>
           </cell>
         </row>
         <row r="12">
@@ -4718,28 +4719,12 @@
             <v>1.2667142201653778E-3</v>
           </cell>
         </row>
-        <row r="13">
-          <cell r="AG13">
-            <v>1.1125652685248788E-2</v>
-          </cell>
-          <cell r="AH13">
-            <v>0.20543141008811813</v>
-          </cell>
-        </row>
         <row r="16">
           <cell r="Y16">
             <v>0.51396946935846444</v>
           </cell>
           <cell r="Z16">
             <v>2.7355760088214132E-3</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="AG17">
-            <v>1.6418388917769666</v>
-          </cell>
-          <cell r="AH17">
-            <v>0.23164910468861188</v>
           </cell>
         </row>
         <row r="20">
@@ -4750,28 +4735,12 @@
             <v>8.9131849042232564E-3</v>
           </cell>
         </row>
-        <row r="21">
-          <cell r="AG21">
-            <v>3.6974788092208</v>
-          </cell>
-          <cell r="AH21">
-            <v>0.47601416888333054</v>
-          </cell>
-        </row>
         <row r="24">
           <cell r="Y24">
             <v>2.6441880127720201</v>
           </cell>
           <cell r="Z24">
             <v>1.4125962771139608E-2</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="AG25">
-            <v>5.2581583200694721</v>
-          </cell>
-          <cell r="AH25">
-            <v>0.82875712549062674</v>
           </cell>
         </row>
         <row r="27">
@@ -4782,28 +4751,12 @@
             <v>3.0856764402689408E-2</v>
           </cell>
         </row>
-        <row r="28">
-          <cell r="AG28">
-            <v>8.9926263591844844</v>
-          </cell>
-          <cell r="AH28">
-            <v>1.3052909818799254</v>
-          </cell>
-        </row>
         <row r="30">
           <cell r="Y30">
             <v>10.325991889146406</v>
           </cell>
           <cell r="Z30">
             <v>6.5981974059936457E-2</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="AG31">
-            <v>9.5082280268323043</v>
-          </cell>
-          <cell r="AH31">
-            <v>1.7092683045581891</v>
           </cell>
         </row>
         <row r="34">
@@ -4814,28 +4767,12 @@
             <v>0.11201750710167138</v>
           </cell>
         </row>
-        <row r="35">
-          <cell r="AG35">
-            <v>3.5751128512312391</v>
-          </cell>
-          <cell r="AH35">
-            <v>1.6845150628351038</v>
-          </cell>
-        </row>
         <row r="37">
           <cell r="Y37">
             <v>23.816066873567554</v>
           </cell>
           <cell r="Z37">
             <v>0.13759790823319112</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="AG38">
-            <v>2.5210171532273193</v>
-          </cell>
-          <cell r="AH38">
-            <v>1.3076850640132609</v>
           </cell>
         </row>
         <row r="40">
@@ -4846,28 +4783,12 @@
             <v>0.15782455273362236</v>
           </cell>
         </row>
-        <row r="41">
-          <cell r="AG41">
-            <v>0.60143930751904229</v>
-          </cell>
-          <cell r="AH41">
-            <v>0.90195738458505448</v>
-          </cell>
-        </row>
         <row r="43">
           <cell r="Y43">
             <v>32.721181560923462</v>
           </cell>
           <cell r="Z43">
             <v>0.16609715597265337</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="AG44">
-            <v>6.6769386443019538</v>
-          </cell>
-          <cell r="AH44">
-            <v>0.91078037198591966</v>
           </cell>
         </row>
         <row r="46">
@@ -4878,28 +4799,12 @@
             <v>0.17637075544473124</v>
           </cell>
         </row>
-        <row r="47">
-          <cell r="AG47">
-            <v>11.113966590277643</v>
-          </cell>
-          <cell r="AH47">
-            <v>1.1975668729731148</v>
-          </cell>
-        </row>
         <row r="49">
           <cell r="Y49">
             <v>46.371019452068559</v>
           </cell>
           <cell r="Z49">
             <v>0.24296486270688972</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="AG50">
-            <v>13.792105763034851</v>
-          </cell>
-          <cell r="AH50">
-            <v>1.2412315132789731</v>
           </cell>
         </row>
         <row r="52">
@@ -4910,28 +4815,12 @@
             <v>0.36095676756397482</v>
           </cell>
         </row>
-        <row r="53">
-          <cell r="AG53">
-            <v>11.358315176506476</v>
-          </cell>
-          <cell r="AH53">
-            <v>1.4517859610795756</v>
-          </cell>
-        </row>
         <row r="55">
           <cell r="Y55">
             <v>68.670750413607593</v>
           </cell>
           <cell r="Z55">
             <v>0.38836770273927967</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="AG56">
-            <v>14.462752797544418</v>
-          </cell>
-          <cell r="AH56">
-            <v>1.9418385862229495</v>
           </cell>
         </row>
         <row r="58">
@@ -4942,28 +4831,12 @@
             <v>0.44771149579712366</v>
           </cell>
         </row>
-        <row r="59">
-          <cell r="AG59">
-            <v>28.330053300207055</v>
-          </cell>
-          <cell r="AH59">
-            <v>2.8402388266383878</v>
-          </cell>
-        </row>
         <row r="61">
           <cell r="Y61">
             <v>100.07115399761372</v>
           </cell>
           <cell r="Z61">
             <v>0.60693388162846851</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="AG62">
-            <v>41.343332028472403</v>
-          </cell>
-          <cell r="AH62">
-            <v>4.0397891565935922</v>
           </cell>
         </row>
         <row r="64">
@@ -4974,28 +4847,12 @@
             <v>0.93372031275444345</v>
           </cell>
         </row>
-        <row r="65">
-          <cell r="AG65">
-            <v>44.783772075614529</v>
-          </cell>
-          <cell r="AH65">
-            <v>4.7710075941316221</v>
-          </cell>
-        </row>
         <row r="67">
           <cell r="Y67">
             <v>176.11865875843083</v>
           </cell>
           <cell r="Z67">
             <v>1.3284958060742038</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="AG68">
-            <v>15.32951848324867</v>
-          </cell>
-          <cell r="AH68">
-            <v>4.0773667157577069</v>
           </cell>
         </row>
         <row r="70">
@@ -5006,28 +4863,12 @@
             <v>1.4733013027815165</v>
           </cell>
         </row>
-        <row r="71">
-          <cell r="AG71">
-            <v>7.4056558378177257</v>
-          </cell>
-          <cell r="AH71">
-            <v>2.55747788992654</v>
-          </cell>
-        </row>
         <row r="73">
           <cell r="Y73">
             <v>218.84623214762186</v>
           </cell>
           <cell r="Z73">
             <v>1.5152230394779262</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="AG74">
-            <v>6.7885433898562955</v>
-          </cell>
-          <cell r="AH74">
-            <v>1.5986131603737967</v>
           </cell>
         </row>
         <row r="76">
@@ -5038,28 +4879,12 @@
             <v>1.5462368369476029</v>
           </cell>
         </row>
-        <row r="77">
-          <cell r="AG77">
-            <v>109.98923129912342</v>
-          </cell>
-          <cell r="AH77">
-            <v>3.2490485062783758</v>
-          </cell>
-        </row>
         <row r="79">
           <cell r="Y79">
             <v>332.5652444551659</v>
           </cell>
           <cell r="Z79">
             <v>3.0805168155550007</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="AG80">
-            <v>5.8007597520409249</v>
-          </cell>
-          <cell r="AH80">
-            <v>1.8876885185255603</v>
           </cell>
         </row>
         <row r="82">
@@ -5070,28 +4895,12 @@
             <v>3.1071655817283692</v>
           </cell>
         </row>
-        <row r="83">
-          <cell r="AG83">
-            <v>18.117517289967918</v>
-          </cell>
-          <cell r="AH83">
-            <v>1.4114442681642989</v>
-          </cell>
-        </row>
         <row r="85">
           <cell r="Y85">
             <v>361.8852084465928</v>
           </cell>
           <cell r="Z85">
             <v>3.1327533703041777</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="AG86">
-            <v>0.70246648635252917</v>
-          </cell>
-          <cell r="AH86">
-            <v>1.2259902068947057</v>
           </cell>
         </row>
         <row r="88">
@@ -5104,7 +4913,7 @@
         </row>
       </sheetData>
       <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2">
+      <sheetData sheetId="2" refreshError="1">
         <row r="12">
           <cell r="H12">
             <v>3.0108969907378196</v>
@@ -5482,7 +5291,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB674F3-CA80-4D41-AE69-30B2094212EF}">
-  <dimension ref="A1:AI89"/>
+  <dimension ref="A1:AJ89"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="9" max="9" width="14.44140625" customWidth="1"/>
@@ -5503,9 +5312,10 @@
     <col min="33" max="33" width="8.88671875" style="31"/>
     <col min="34" max="34" width="8.88671875" style="30"/>
     <col min="35" max="35" width="8.88671875" style="29"/>
+    <col min="36" max="36" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>64</v>
       </c>
@@ -5527,8 +5337,11 @@
       <c r="AB1" s="3">
         <v>1.3621000000000001E-22</v>
       </c>
+      <c r="AJ1" t="s">
+        <v>141</v>
+      </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="N2" s="33" t="s">
         <v>136</v>
       </c>
@@ -5548,7 +5361,7 @@
       <c r="X2" s="59"/>
       <c r="AA2" s="12"/>
     </row>
-    <row r="3" spans="1:35" ht="16.8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" ht="16.8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -5652,8 +5465,9 @@
       <c r="AI3" s="29" t="s">
         <v>118</v>
       </c>
+      <c r="AJ3" s="4"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -5739,8 +5553,9 @@
       <c r="Z4" s="32">
         <v>0</v>
       </c>
+      <c r="AJ4" s="4"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -5831,7 +5646,7 @@
         <v>3243.9999999012798</v>
       </c>
       <c r="AB5" s="4">
-        <f t="shared" ref="AB5:AB36" si="2">(0.000304*199000000000000000)*EXP(-(5580-680)/(1.987*(C5+273)))</f>
+        <f>(0.000304*199000000000000000)*EXP(-(5580-680)/(1.987*(C5+273)))</f>
         <v>15113410716.254675</v>
       </c>
       <c r="AC5" s="4">
@@ -5846,8 +5661,9 @@
         <f>(((X5/W5)*AD5)^2+(AD5*0.1)^2)^0.5</f>
         <v>0.18250619135834925</v>
       </c>
+      <c r="AJ5" s="4"/>
     </row>
-    <row r="6" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -5938,7 +5754,7 @@
         <v>3256.0000001918525</v>
       </c>
       <c r="AB6" s="15">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="AB6:AB69" si="2">(0.000304*199000000000000000)*EXP(-(5580-680)/(1.987*(C6+273)))</f>
         <v>15113410716.254675</v>
       </c>
       <c r="AC6" s="15">
@@ -5963,8 +5779,9 @@
       </c>
       <c r="AH6" s="37"/>
       <c r="AI6" s="36"/>
+      <c r="AJ6" s="15"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -6032,8 +5849,9 @@
       <c r="AF7" s="30" t="s">
         <v>98</v>
       </c>
+      <c r="AJ7" s="4"/>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -6102,8 +5920,9 @@
       <c r="AF8" s="30" t="s">
         <v>98</v>
       </c>
+      <c r="AJ8" s="4"/>
     </row>
-    <row r="9" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>22</v>
       </c>
@@ -6218,8 +6037,12 @@
         <f>(X9^2+AG9^2+AG10^2)^0.5</f>
         <v>0.23714864603814678</v>
       </c>
+      <c r="AJ9" s="7">
+        <f>0.2*AF9/($B$89-Y9)</f>
+        <v>4.7699852169037771E-4</v>
+      </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -6335,8 +6158,12 @@
         <f>(X10^2+AG11^2)^0.5</f>
         <v>0.15764617940935433</v>
       </c>
+      <c r="AJ10" s="4">
+        <f t="shared" ref="AJ10:AJ73" si="11">0.2*AF10/($B$89-Y10)</f>
+        <v>4.3800440077673041E-4</v>
+      </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -6452,8 +6279,12 @@
         <f>(X11^2+AG12^2)^0.5</f>
         <v>0.15764569011306748</v>
       </c>
+      <c r="AJ11" s="4">
+        <f t="shared" si="11"/>
+        <v>4.35674398311148E-4</v>
+      </c>
     </row>
-    <row r="12" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>15</v>
       </c>
@@ -6571,8 +6402,12 @@
       </c>
       <c r="AH12" s="37"/>
       <c r="AI12" s="36"/>
+      <c r="AJ12" s="15">
+        <f t="shared" si="11"/>
+        <v>4.3360844897602675E-4</v>
+      </c>
     </row>
-    <row r="13" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>24</v>
       </c>
@@ -6687,8 +6522,12 @@
         <f>(X13^2+AG13^2+AG14^2)^0.5</f>
         <v>0.20543141008811813</v>
       </c>
+      <c r="AJ13" s="7">
+        <f t="shared" si="11"/>
+        <v>4.3178248146681674E-4</v>
+      </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -6804,8 +6643,12 @@
         <f>(X14^2+AG15^2)^0.5</f>
         <v>0.13169845404220318</v>
       </c>
+      <c r="AJ14" s="4">
+        <f t="shared" si="11"/>
+        <v>3.3524324582815274E-4</v>
+      </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -6921,8 +6764,12 @@
         <f>(X15^2+AG16^2)^0.5</f>
         <v>0.13169786943406672</v>
       </c>
+      <c r="AJ15" s="4">
+        <f t="shared" si="11"/>
+        <v>3.3348969000861954E-4</v>
+      </c>
     </row>
-    <row r="16" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>15</v>
       </c>
@@ -7040,8 +6887,12 @@
       </c>
       <c r="AH16" s="37"/>
       <c r="AI16" s="36"/>
+      <c r="AJ16" s="15">
+        <f t="shared" si="11"/>
+        <v>3.3192215842940833E-4</v>
+      </c>
     </row>
-    <row r="17" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>26</v>
       </c>
@@ -7156,8 +7007,12 @@
         <f>(X17^2+AG17^2+AG18^2)^0.5</f>
         <v>0.23164910468861188</v>
       </c>
+      <c r="AJ17" s="7">
+        <f t="shared" si="11"/>
+        <v>3.3085599086943855E-4</v>
+      </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -7273,8 +7128,12 @@
         <f>(X18^2+AG19^2)^0.5</f>
         <v>0.19038252257887187</v>
       </c>
+      <c r="AJ18" s="4">
+        <f t="shared" si="11"/>
+        <v>5.5818088815047116E-4</v>
+      </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -7390,8 +7249,12 @@
         <f>(X19^2+AG20^2)^0.5</f>
         <v>0.19038209075713142</v>
       </c>
+      <c r="AJ19" s="4">
+        <f t="shared" si="11"/>
+        <v>5.5511440316792125E-4</v>
+      </c>
     </row>
-    <row r="20" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>15</v>
       </c>
@@ -7509,8 +7372,12 @@
       </c>
       <c r="AH20" s="37"/>
       <c r="AI20" s="36"/>
+      <c r="AJ20" s="15">
+        <f t="shared" si="11"/>
+        <v>5.5257097067950233E-4</v>
+      </c>
     </row>
-    <row r="21" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>28</v>
       </c>
@@ -7625,8 +7492,12 @@
         <f>(X21^2+AG21^2+AG22^2)^0.5</f>
         <v>0.47601416888333054</v>
       </c>
+      <c r="AJ21" s="7">
+        <f t="shared" si="11"/>
+        <v>5.5094288008748435E-4</v>
+      </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -7742,8 +7613,12 @@
         <f>(X22^2+AG23^2)^0.5</f>
         <v>0.43614760153263687</v>
       </c>
+      <c r="AJ22" s="4">
+        <f t="shared" si="11"/>
+        <v>1.3968650441363137E-3</v>
+      </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -7859,8 +7734,12 @@
         <f>(X23^2+AG24^2)^0.5</f>
         <v>0.43614731546863977</v>
       </c>
+      <c r="AJ23" s="4">
+        <f t="shared" si="11"/>
+        <v>1.3882811077594425E-3</v>
+      </c>
     </row>
-    <row r="24" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
         <v>15</v>
       </c>
@@ -7978,8 +7857,12 @@
       </c>
       <c r="AH24" s="37"/>
       <c r="AI24" s="36"/>
+      <c r="AJ24" s="15">
+        <f t="shared" si="11"/>
+        <v>1.3817700916540375E-3</v>
+      </c>
     </row>
-    <row r="25" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>30</v>
       </c>
@@ -8094,8 +7977,12 @@
         <f>(X25^2+AG25^2+AG26^2)^0.5</f>
         <v>0.82875712549062674</v>
       </c>
+      <c r="AJ25" s="7">
+        <f t="shared" si="11"/>
+        <v>1.3808861007793755E-3</v>
+      </c>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>15</v>
       </c>
@@ -8211,8 +8098,12 @@
         <f>(X26^2+AG27^2)^0.5</f>
         <v>0.70417474311307271</v>
       </c>
+      <c r="AJ26" s="4">
+        <f t="shared" si="11"/>
+        <v>2.2793061643927616E-3</v>
+      </c>
     </row>
-    <row r="27" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
         <v>15</v>
       </c>
@@ -8330,8 +8221,12 @@
       </c>
       <c r="AH27" s="37"/>
       <c r="AI27" s="36"/>
+      <c r="AJ27" s="15">
+        <f t="shared" si="11"/>
+        <v>2.2650089121634539E-3</v>
+      </c>
     </row>
-    <row r="28" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>32</v>
       </c>
@@ -8446,8 +8341,12 @@
         <f>(X28^2+AG28^2+AG29^2)^0.5</f>
         <v>1.3052909818799254</v>
       </c>
+      <c r="AJ28" s="7">
+        <f t="shared" si="11"/>
+        <v>2.2728876629290623E-3</v>
+      </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -8563,8 +8462,12 @@
         <f>(X29^2+AG30^2)^0.5</f>
         <v>1.0975074622962924</v>
       </c>
+      <c r="AJ29" s="4">
+        <f t="shared" si="11"/>
+        <v>3.5950255625324633E-3</v>
+      </c>
     </row>
-    <row r="30" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="13" t="s">
         <v>15</v>
       </c>
@@ -8682,8 +8585,12 @@
       </c>
       <c r="AH30" s="37"/>
       <c r="AI30" s="36"/>
+      <c r="AJ30" s="15">
+        <f t="shared" si="11"/>
+        <v>3.5728738131667781E-3</v>
+      </c>
     </row>
-    <row r="31" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>34</v>
       </c>
@@ -8798,8 +8705,12 @@
         <f>(X31^2+AG31^2+AG32^2)^0.5</f>
         <v>1.7092683045581891</v>
       </c>
+      <c r="AJ31" s="7">
+        <f t="shared" si="11"/>
+        <v>3.599169382292663E-3</v>
+      </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -8915,8 +8826,12 @@
         <f>(X32^2+AG33^2)^0.5</f>
         <v>1.3072431852381001</v>
       </c>
+      <c r="AJ32" s="4">
+        <f t="shared" si="11"/>
+        <v>4.3550256504461858E-3</v>
+      </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -9032,8 +8947,12 @@
         <f>(X33^2+AG34^2)^0.5</f>
         <v>1.3072426342175432</v>
       </c>
+      <c r="AJ33" s="4">
+        <f t="shared" si="11"/>
+        <v>4.3273516170790503E-3</v>
+      </c>
     </row>
-    <row r="34" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="13" t="s">
         <v>15</v>
       </c>
@@ -9151,8 +9070,12 @@
       </c>
       <c r="AH34" s="37"/>
       <c r="AI34" s="36"/>
+      <c r="AJ34" s="15">
+        <f t="shared" si="11"/>
+        <v>4.3072493069532579E-3</v>
+      </c>
     </row>
-    <row r="35" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>36</v>
       </c>
@@ -9267,8 +9190,12 @@
         <f>(X35^2+AG35^2+AG36^2)^0.5</f>
         <v>1.6845150628351038</v>
       </c>
+      <c r="AJ35" s="7">
+        <f t="shared" si="11"/>
+        <v>4.3296491080493027E-3</v>
+      </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>15</v>
       </c>
@@ -9303,7 +9230,7 @@
         <v>190.748741</v>
       </c>
       <c r="M36" s="32">
-        <f t="shared" ref="M36:M67" si="11">L36/K36</f>
+        <f t="shared" ref="M36:M67" si="12">L36/K36</f>
         <v>2.3920660223057059E-2</v>
       </c>
       <c r="N36" s="33">
@@ -9384,8 +9311,12 @@
         <f>(X36^2+AG37^2)^0.5</f>
         <v>1.0593981376639101</v>
       </c>
+      <c r="AJ36" s="4">
+        <f t="shared" si="11"/>
+        <v>3.5406260578083226E-3</v>
+      </c>
     </row>
-    <row r="37" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="13" t="s">
         <v>15</v>
       </c>
@@ -9420,7 +9351,7 @@
         <v>131.15876399999999</v>
       </c>
       <c r="M37" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.6455594470004564E-2</v>
       </c>
       <c r="N37" s="40">
@@ -9474,11 +9405,11 @@
         <v>0.13759790823319112</v>
       </c>
       <c r="AA37" s="13">
-        <f t="shared" ref="AA37:AA68" si="12">((I37-I36)*24*3600)-(5*60)</f>
+        <f t="shared" ref="AA37:AA68" si="13">((I37-I36)*24*3600)-(5*60)</f>
         <v>3246.999999973923</v>
       </c>
       <c r="AB37" s="15">
-        <f t="shared" ref="AB37:AB68" si="13">(0.000304*199000000000000000)*EXP(-(5580-680)/(1.987*(C37+273)))</f>
+        <f t="shared" si="2"/>
         <v>14820423493.51034</v>
       </c>
       <c r="AC37" s="15">
@@ -9503,8 +9434,12 @@
       </c>
       <c r="AH37" s="37"/>
       <c r="AI37" s="36"/>
+      <c r="AJ37" s="15">
+        <f t="shared" si="11"/>
+        <v>3.5163577075384999E-3</v>
+      </c>
     </row>
-    <row r="38" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>38</v>
       </c>
@@ -9539,7 +9474,7 @@
         <v>13180.380721</v>
       </c>
       <c r="M38" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.6474123435434649</v>
       </c>
       <c r="N38" s="51">
@@ -9593,11 +9528,11 @@
         <v>0.1578202947185828</v>
       </c>
       <c r="AA38" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7203.9999996079132</v>
       </c>
       <c r="AB38" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>673118247451.83813</v>
       </c>
       <c r="AC38" s="7"/>
@@ -9619,8 +9554,12 @@
         <f>(X38^2+AG38^2+AG39^2)^0.5</f>
         <v>1.3076850640132609</v>
       </c>
+      <c r="AJ38" s="7">
+        <f t="shared" si="11"/>
+        <v>3.532052974708118E-3</v>
+      </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -9655,7 +9594,7 @@
         <v>140.78924799999999</v>
       </c>
       <c r="M39" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.7679161305129004E-2</v>
       </c>
       <c r="N39" s="33">
@@ -9709,11 +9648,11 @@
         <v>0.15782298595871372</v>
       </c>
       <c r="AA39">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3248.0000002076849</v>
       </c>
       <c r="AB39" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21229668396.533699</v>
       </c>
       <c r="AC39" s="4">
@@ -9736,8 +9675,12 @@
         <f>(X39^2+AG40^2)^0.5</f>
         <v>0.76272035539089955</v>
       </c>
+      <c r="AJ39" s="4">
+        <f t="shared" si="11"/>
+        <v>2.5595856769056275E-3</v>
+      </c>
     </row>
-    <row r="40" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
         <v>15</v>
       </c>
@@ -9772,7 +9715,7 @@
         <v>97.889358999999999</v>
       </c>
       <c r="M40" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.2311764018351358E-2</v>
       </c>
       <c r="N40" s="40">
@@ -9826,11 +9769,11 @@
         <v>0.15782455273362236</v>
       </c>
       <c r="AA40" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3261.999999708496</v>
       </c>
       <c r="AB40" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14820423493.51034</v>
       </c>
       <c r="AC40" s="15">
@@ -9855,8 +9798,12 @@
       </c>
       <c r="AH40" s="37"/>
       <c r="AI40" s="36"/>
+      <c r="AJ40" s="15">
+        <f t="shared" si="11"/>
+        <v>2.5419130218398453E-3</v>
+      </c>
     </row>
-    <row r="41" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>40</v>
       </c>
@@ -9891,7 +9838,7 @@
         <v>8344.7624510000005</v>
       </c>
       <c r="M41" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.0366679890748502</v>
       </c>
       <c r="N41" s="51">
@@ -9945,11 +9892,11 @@
         <v>0.16609476158757014</v>
       </c>
       <c r="AA41" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8417.0000002719462</v>
       </c>
       <c r="AB41" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>567698892732.06018</v>
       </c>
       <c r="AC41" s="7"/>
@@ -9971,8 +9918,12 @@
         <f>(X41^2+AG41^2+AG42^2)^0.5</f>
         <v>0.90195738458505448</v>
       </c>
+      <c r="AJ41" s="7">
+        <f t="shared" si="11"/>
+        <v>2.5446869026430007E-3</v>
+      </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -10007,7 +9958,7 @@
         <v>91.577528999999998</v>
       </c>
       <c r="M42" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.1461409771736293E-2</v>
       </c>
       <c r="N42" s="33">
@@ -10061,11 +10012,11 @@
         <v>0.16609619784296553</v>
       </c>
       <c r="AA42">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3232.9999998444691</v>
       </c>
       <c r="AB42" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21284198349.863953</v>
       </c>
       <c r="AC42" s="4">
@@ -10088,8 +10039,12 @@
         <f>(X42^2+AG43^2)^0.5</f>
         <v>0.47865045453007582</v>
       </c>
+      <c r="AJ42" s="4">
+        <f t="shared" si="11"/>
+        <v>1.5940410215775911E-3</v>
+      </c>
     </row>
-    <row r="43" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
         <v>15</v>
       </c>
@@ -10124,7 +10079,7 @@
         <v>65.659137000000001</v>
       </c>
       <c r="M43" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>8.2206658296260348E-3</v>
       </c>
       <c r="N43" s="40">
@@ -10178,11 +10133,11 @@
         <v>0.16609715597265337</v>
       </c>
       <c r="AA43" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3243.9999999012798</v>
       </c>
       <c r="AB43" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14820423493.51034</v>
       </c>
       <c r="AC43" s="15">
@@ -10207,8 +10162,12 @@
       </c>
       <c r="AH43" s="37"/>
       <c r="AI43" s="36"/>
+      <c r="AJ43" s="15">
+        <f t="shared" si="11"/>
+        <v>1.5831347156110699E-3</v>
+      </c>
     </row>
-    <row r="44" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>34</v>
       </c>
@@ -10243,7 +10202,7 @@
         <v>9069.5688850000006</v>
       </c>
       <c r="M44" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.1301704647482853</v>
       </c>
       <c r="N44" s="51">
@@ -10297,11 +10256,11 @@
         <v>0.17636623854305344</v>
       </c>
       <c r="AA44" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6010.0000002421439</v>
       </c>
       <c r="AB44" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>819642883937.08691</v>
       </c>
       <c r="AC44" s="7"/>
@@ -10323,8 +10282,12 @@
         <f>(X44^2+AG44^2+AG45^2)^0.5</f>
         <v>0.91078037198591966</v>
       </c>
+      <c r="AJ44" s="7">
+        <f t="shared" si="11"/>
+        <v>1.5857820948319661E-3</v>
+      </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -10359,7 +10322,7 @@
         <v>139.97025600000001</v>
       </c>
       <c r="M45" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.7519720065460636E-2</v>
       </c>
       <c r="N45" s="33">
@@ -10413,11 +10376,11 @@
         <v>0.17636909346652901</v>
       </c>
       <c r="AA45">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3235.9999999171123</v>
       </c>
       <c r="AB45" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>20850882042.20224</v>
       </c>
       <c r="AC45" s="4">
@@ -10440,8 +10403,12 @@
         <f>(X45^2+AG46^2)^0.5</f>
         <v>0.77259174362924954</v>
       </c>
+      <c r="AJ45" s="4">
+        <f t="shared" si="11"/>
+        <v>2.6159081715888145E-3</v>
+      </c>
     </row>
-    <row r="46" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="13" t="s">
         <v>15</v>
       </c>
@@ -10476,7 +10443,7 @@
         <v>99.067865999999995</v>
       </c>
       <c r="M46" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.2412284869413011E-2</v>
       </c>
       <c r="N46" s="40">
@@ -10530,11 +10497,11 @@
         <v>0.17637075544473124</v>
       </c>
       <c r="AA46" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3254.9999999580905</v>
       </c>
       <c r="AB46" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14820423493.51034</v>
       </c>
       <c r="AC46" s="15">
@@ -10559,8 +10526,12 @@
       </c>
       <c r="AH46" s="37"/>
       <c r="AI46" s="36"/>
+      <c r="AJ46" s="15">
+        <f t="shared" si="11"/>
+        <v>2.5982338845396947E-3</v>
+      </c>
     </row>
-    <row r="47" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>42</v>
       </c>
@@ -10595,7 +10566,7 @@
         <v>23839.943576000001</v>
       </c>
       <c r="M47" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.9998408555493086</v>
       </c>
       <c r="N47" s="51">
@@ -10649,11 +10620,11 @@
         <v>0.24296035403146912</v>
       </c>
       <c r="AA47" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>9610.0000000325963</v>
       </c>
       <c r="AB47" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>819028030197.81494</v>
       </c>
       <c r="AC47" s="7"/>
@@ -10675,8 +10646,12 @@
         <f>(X47^2+AG47^2+AG48^2)^0.5</f>
         <v>1.1975668729731148</v>
       </c>
+      <c r="AJ47" s="7">
+        <f t="shared" si="11"/>
+        <v>2.6304072251704682E-3</v>
+      </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -10711,7 +10686,7 @@
         <v>159.47943699999999</v>
       </c>
       <c r="M48" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.9890146286856435E-2</v>
       </c>
       <c r="N48" s="33">
@@ -10765,11 +10740,11 @@
         <v>0.2429632285099336</v>
       </c>
       <c r="AA48">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3243.0000002961606</v>
       </c>
       <c r="AB48" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>20530257565.267223</v>
       </c>
       <c r="AC48" s="4">
@@ -10792,8 +10767,12 @@
         <f>(X48^2+AG49^2)^0.5</f>
         <v>0.89963645071218012</v>
       </c>
+      <c r="AJ48" s="4">
+        <f t="shared" si="11"/>
+        <v>3.0983566313777505E-3</v>
+      </c>
     </row>
-    <row r="49" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="13" t="s">
         <v>15</v>
       </c>
@@ -10828,7 +10807,7 @@
         <v>113.643236</v>
       </c>
       <c r="M49" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.4184670081558371E-2</v>
       </c>
       <c r="N49" s="40">
@@ -10882,11 +10861,11 @@
         <v>0.24296486270688972</v>
       </c>
       <c r="AA49" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3251.9999998854473</v>
       </c>
       <c r="AB49" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14820423493.51034</v>
       </c>
       <c r="AC49" s="15">
@@ -10911,8 +10890,12 @@
       </c>
       <c r="AH49" s="37"/>
       <c r="AI49" s="36"/>
+      <c r="AJ49" s="15">
+        <f t="shared" si="11"/>
+        <v>3.0777509819657901E-3</v>
+      </c>
     </row>
-    <row r="50" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>43</v>
       </c>
@@ -10947,7 +10930,7 @@
         <v>35191.554955</v>
       </c>
       <c r="M50" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4.4772013328561302</v>
       </c>
       <c r="N50" s="51">
@@ -11001,11 +10984,11 @@
         <v>0.36095376581264893</v>
       </c>
       <c r="AA50" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>13211.99999966193</v>
       </c>
       <c r="AB50" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>818413423360.28638</v>
       </c>
       <c r="AC50" s="7"/>
@@ -11027,8 +11010,12 @@
         <f>(X50^2+AG50^2+AG51^2)^0.5</f>
         <v>1.2412315132789731</v>
       </c>
+      <c r="AJ50" s="7">
+        <f t="shared" si="11"/>
+        <v>3.1436764287610733E-3</v>
+      </c>
     </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>15</v>
       </c>
@@ -11063,7 +11050,7 @@
         <v>147.12985499999999</v>
       </c>
       <c r="M51" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.8437441378507453E-2</v>
       </c>
       <c r="N51" s="33">
@@ -11117,11 +11104,11 @@
         <v>0.36095566949229785</v>
       </c>
       <c r="AA51">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3251.0000002803281</v>
       </c>
       <c r="AB51" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>20636718843.809963</v>
       </c>
       <c r="AC51" s="4">
@@ -11144,8 +11131,12 @@
         <f>(X51^2+AG52^2)^0.5</f>
         <v>0.81243758667193111</v>
       </c>
+      <c r="AJ51" s="4">
+        <f t="shared" si="11"/>
+        <v>2.8614865554023048E-3</v>
+      </c>
     </row>
-    <row r="52" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>15</v>
       </c>
@@ -11180,7 +11171,7 @@
         <v>106.162623</v>
       </c>
       <c r="M52" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.3264856784819101E-2</v>
       </c>
       <c r="N52" s="40">
@@ -11234,11 +11225,11 @@
         <v>0.36095676756397482</v>
       </c>
       <c r="AA52" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3345.0000002514571</v>
       </c>
       <c r="AB52" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14820423493.51034</v>
       </c>
       <c r="AC52" s="15">
@@ -11263,8 +11254,12 @@
       </c>
       <c r="AH52" s="37"/>
       <c r="AI52" s="36"/>
+      <c r="AJ52" s="15">
+        <f t="shared" si="11"/>
+        <v>2.84203300966638E-3</v>
+      </c>
     </row>
-    <row r="53" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>44</v>
       </c>
@@ -11299,7 +11294,7 @@
         <v>18313.281958</v>
       </c>
       <c r="M53" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.3040893445443933</v>
       </c>
       <c r="N53" s="51">
@@ -11353,11 +11348,11 @@
         <v>0.38836200013050004</v>
       </c>
       <c r="AA53" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6034.9999997997656</v>
       </c>
       <c r="AB53" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>947540846265.11804</v>
       </c>
       <c r="AC53" s="7"/>
@@ -11379,8 +11374,12 @@
         <f>(X53^2+AG53^2+AG54^2)^0.5</f>
         <v>1.4517859610795756</v>
       </c>
+      <c r="AJ53" s="7">
+        <f t="shared" si="11"/>
+        <v>2.8670475067975542E-3</v>
+      </c>
     </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>15</v>
       </c>
@@ -11415,7 +11414,7 @@
         <v>212.99306000000001</v>
       </c>
       <c r="M54" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.6631464558309538E-2</v>
       </c>
       <c r="N54" s="33">
@@ -11469,11 +11468,11 @@
         <v>0.38836578658889187</v>
       </c>
       <c r="AA54">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3253.0000001192093</v>
       </c>
       <c r="AB54" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21175243091.75367</v>
       </c>
       <c r="AC54" s="4">
@@ -11496,8 +11495,12 @@
         <f>(X54^2+AG55^2)^0.5</f>
         <v>1.1946099660675888</v>
       </c>
+      <c r="AJ54" s="4">
+        <f t="shared" si="11"/>
+        <v>4.2755413464405983E-3</v>
+      </c>
     </row>
-    <row r="55" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
         <v>15</v>
       </c>
@@ -11532,7 +11535,7 @@
         <v>146.14432300000001</v>
       </c>
       <c r="M55" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.8289473562159604E-2</v>
       </c>
       <c r="N55" s="40">
@@ -11586,11 +11589,11 @@
         <v>0.38836770273927967</v>
       </c>
       <c r="AA55" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3258.9999996358529</v>
       </c>
       <c r="AB55" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14778922909.376841</v>
       </c>
       <c r="AC55" s="15">
@@ -11615,8 +11618,12 @@
       </c>
       <c r="AH55" s="37"/>
       <c r="AI55" s="36"/>
+      <c r="AJ55" s="15">
+        <f t="shared" si="11"/>
+        <v>4.2463440175619363E-3</v>
+      </c>
     </row>
-    <row r="56" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>46</v>
       </c>
@@ -11651,7 +11658,7 @@
         <v>27246.357620999999</v>
       </c>
       <c r="M56" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.4395980307327374</v>
       </c>
       <c r="N56" s="51">
@@ -11705,11 +11712,11 @@
         <v>0.44770285484672678</v>
       </c>
       <c r="AA56" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6054.0000004693866</v>
       </c>
       <c r="AB56" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>1015811335703.1714</v>
       </c>
       <c r="AC56" s="7"/>
@@ -11731,8 +11738,12 @@
         <f>(X56^2+AG56^2+AG57^2)^0.5</f>
         <v>1.9418385862229495</v>
       </c>
+      <c r="AJ56" s="7">
+        <f t="shared" si="11"/>
+        <v>4.3145012739194376E-3</v>
+      </c>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>15</v>
       </c>
@@ -11767,7 +11778,7 @@
         <v>277.42042500000002</v>
       </c>
       <c r="M57" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.4759009704159752E-2</v>
       </c>
       <c r="N57" s="33">
@@ -11821,11 +11832,11 @@
         <v>0.44770878438761169</v>
       </c>
       <c r="AA57">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3250.9999996516854</v>
       </c>
       <c r="AB57" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21448417322.985222</v>
       </c>
       <c r="AC57" s="4">
@@ -11848,8 +11859,12 @@
         <f>(X57^2+AG58^2)^0.5</f>
         <v>1.514607937031456</v>
       </c>
+      <c r="AJ57" s="4">
+        <f t="shared" si="11"/>
+        <v>5.53659226754105E-3</v>
+      </c>
     </row>
-    <row r="58" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="13" t="s">
         <v>15</v>
       </c>
@@ -11884,7 +11899,7 @@
         <v>182.861977</v>
       </c>
       <c r="M58" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.2896186720069697E-2</v>
       </c>
       <c r="N58" s="40">
@@ -11938,11 +11953,11 @@
         <v>0.44771149579712366</v>
       </c>
       <c r="AA58" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3259.0000002644956</v>
       </c>
       <c r="AB58" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14862012522.468014</v>
       </c>
       <c r="AC58" s="15">
@@ -11967,8 +11982,12 @@
       </c>
       <c r="AH58" s="37"/>
       <c r="AI58" s="36"/>
+      <c r="AJ58" s="15">
+        <f t="shared" si="11"/>
+        <v>5.4972525614531047E-3</v>
+      </c>
     </row>
-    <row r="59" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>48</v>
       </c>
@@ -12003,7 +12022,7 @@
         <v>48106.0481</v>
       </c>
       <c r="M59" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.0875545156801714</v>
       </c>
       <c r="N59" s="51">
@@ -12057,11 +12076,11 @@
         <v>0.60691895689420272</v>
       </c>
       <c r="AA59" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6039.0000001061708</v>
       </c>
       <c r="AB59" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>1158126673954.6372</v>
       </c>
       <c r="AC59" s="7"/>
@@ -12083,8 +12102,12 @@
         <f>(X59^2+AG59^2+AG60^2)^0.5</f>
         <v>2.8402388266383878</v>
       </c>
+      <c r="AJ59" s="7">
+        <f t="shared" si="11"/>
+        <v>5.6805381502192335E-3</v>
+      </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>15</v>
       </c>
@@ -12119,7 +12142,7 @@
         <v>407.594494</v>
       </c>
       <c r="M60" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>5.135671121945698E-2</v>
       </c>
       <c r="N60" s="33">
@@ -12173,11 +12196,11 @@
         <v>0.60692911272621397</v>
       </c>
       <c r="AA60">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3252.9999994905666</v>
       </c>
       <c r="AB60" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21229668396.533699</v>
       </c>
       <c r="AC60" s="4">
@@ -12200,8 +12223,12 @@
         <f>(X60^2+AG61^2)^0.5</f>
         <v>2.3674917601093637</v>
       </c>
+      <c r="AJ60" s="4">
+        <f t="shared" si="11"/>
+        <v>8.9880137445914454E-3</v>
+      </c>
     </row>
-    <row r="61" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="13" t="s">
         <v>15</v>
       </c>
@@ -12236,7 +12263,7 @@
         <v>274.76486199999999</v>
       </c>
       <c r="M61" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.4625879024406163E-2</v>
       </c>
       <c r="N61" s="40">
@@ -12290,11 +12317,11 @@
         <v>0.60693388162846851</v>
       </c>
       <c r="AA61" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3253.0000001192093</v>
       </c>
       <c r="AB61" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14778922909.376841</v>
       </c>
       <c r="AC61" s="15">
@@ -12319,8 +12346,12 @@
       </c>
       <c r="AH61" s="37"/>
       <c r="AI61" s="36"/>
+      <c r="AJ61" s="15">
+        <f t="shared" si="11"/>
+        <v>8.9274675309021344E-3</v>
+      </c>
     </row>
-    <row r="62" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>50</v>
       </c>
@@ -12355,7 +12386,7 @@
         <v>80392.342027999999</v>
       </c>
       <c r="M62" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>10.155383812900524</v>
       </c>
       <c r="N62" s="51">
@@ -12409,11 +12440,11 @@
         <v>0.9337014292527186</v>
       </c>
       <c r="AA62" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6036.0000000335276</v>
       </c>
       <c r="AB62" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>1309661143940.5559</v>
       </c>
       <c r="AC62" s="7"/>
@@ -12435,8 +12466,12 @@
         <f>(X62^2+AG62^2+AG63^2)^0.5</f>
         <v>4.0397891565935922</v>
       </c>
+      <c r="AJ62" s="7">
+        <f t="shared" si="11"/>
+        <v>9.4906680309057769E-3</v>
+      </c>
     </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>15</v>
       </c>
@@ -12471,7 +12506,7 @@
         <v>550.30167900000004</v>
       </c>
       <c r="M63" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.9650794988312101E-2</v>
       </c>
       <c r="N63" s="33">
@@ -12525,11 +12560,11 @@
         <v>0.93371442998652776</v>
       </c>
       <c r="AA63">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3259.9999998696148</v>
       </c>
       <c r="AB63" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21393572690.89529</v>
       </c>
       <c r="AC63" s="4">
@@ -12552,8 +12587,12 @@
         <f>(X63^2+AG64^2)^0.5</f>
         <v>3.1955369051332481</v>
       </c>
+      <c r="AJ63" s="4">
+        <f t="shared" si="11"/>
+        <v>1.2954676425963815E-2</v>
+      </c>
     </row>
-    <row r="64" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="13" t="s">
         <v>15</v>
       </c>
@@ -12588,7 +12627,7 @@
         <v>366.180724</v>
       </c>
       <c r="M64" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4.6249619510703797E-2</v>
       </c>
       <c r="N64" s="40">
@@ -12642,11 +12681,11 @@
         <v>0.93372031275444345</v>
       </c>
       <c r="AA64" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3260.0000004982576</v>
       </c>
       <c r="AB64" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14778922909.376841</v>
       </c>
       <c r="AC64" s="15">
@@ -12671,8 +12710,12 @@
       </c>
       <c r="AH64" s="37"/>
       <c r="AI64" s="36"/>
+      <c r="AJ64" s="15">
+        <f t="shared" si="11"/>
+        <v>1.2867371812923911E-2</v>
+      </c>
     </row>
-    <row r="65" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>52</v>
       </c>
@@ -12707,7 +12750,7 @@
         <v>103104.06658699999</v>
       </c>
       <c r="M65" s="50">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>13.047944407146744</v>
       </c>
       <c r="N65" s="51">
@@ -12761,11 +12804,11 @@
         <v>1.3284792633498297</v>
       </c>
       <c r="AA65" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6033.9999995660037</v>
       </c>
       <c r="AB65" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>1429163650537.043</v>
       </c>
       <c r="AC65" s="7"/>
@@ -12787,8 +12830,12 @@
         <f>(X65^2+AG65^2+AG66^2)^0.5</f>
         <v>4.7710075941316221</v>
       </c>
+      <c r="AJ65" s="7">
+        <f t="shared" si="11"/>
+        <v>1.4034401867917531E-2</v>
+      </c>
     </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>15</v>
       </c>
@@ -12823,7 +12870,7 @@
         <v>595.17753200000004</v>
       </c>
       <c r="M66" s="32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>7.5428396605945427E-2</v>
       </c>
       <c r="N66" s="33">
@@ -12877,11 +12924,11 @@
         <v>1.3284907567411941</v>
       </c>
       <c r="AA66">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3251.0000002803281</v>
       </c>
       <c r="AB66" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>21668848446.899525</v>
       </c>
       <c r="AC66" s="4">
@@ -12904,8 +12951,12 @@
         <f>(X66^2+AG67^2)^0.5</f>
         <v>3.4143882486594994</v>
       </c>
+      <c r="AJ66" s="4">
+        <f t="shared" si="11"/>
+        <v>1.5156849610569867E-2</v>
+      </c>
     </row>
-    <row r="67" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="13" t="s">
         <v>15</v>
       </c>
@@ -12940,7 +12991,7 @@
         <v>390.64191699999998</v>
       </c>
       <c r="M67" s="39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4.9395022247635686E-2</v>
       </c>
       <c r="N67" s="40">
@@ -12994,11 +13045,11 @@
         <v>1.3284958060742038</v>
       </c>
       <c r="AA67" s="13">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3269.0000000875443</v>
       </c>
       <c r="AB67" s="15">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>14778922909.376841</v>
       </c>
       <c r="AC67" s="15">
@@ -13023,8 +13074,12 @@
       </c>
       <c r="AH67" s="37"/>
       <c r="AI67" s="36"/>
+      <c r="AJ67" s="15">
+        <f t="shared" si="11"/>
+        <v>1.5053758132179672E-2</v>
+      </c>
     </row>
-    <row r="68" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>54</v>
       </c>
@@ -13113,11 +13168,11 @@
         <v>1.4732940838948989</v>
       </c>
       <c r="AA68" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>6037.9999998724088</v>
       </c>
       <c r="AB68" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="2"/>
         <v>1232761495022.8789</v>
       </c>
       <c r="AC68" s="7"/>
@@ -13139,8 +13194,12 @@
         <f>(X68^2+AG68^2+AG69^2)^0.5</f>
         <v>4.0773667157577069</v>
       </c>
+      <c r="AJ68" s="7">
+        <f t="shared" si="11"/>
+        <v>1.5980136394931378E-2</v>
+      </c>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>15</v>
       </c>
@@ -13233,7 +13292,7 @@
         <v>3261.999999708496</v>
       </c>
       <c r="AB69" s="4">
-        <f t="shared" ref="AB69:AB88" si="22">(0.000304*199000000000000000)*EXP(-(5580-680)/(1.987*(C69+273)))</f>
+        <f t="shared" si="2"/>
         <v>22681815520.592377</v>
       </c>
       <c r="AC69" s="4">
@@ -13256,8 +13315,12 @@
         <f>(X69^2+AG70^2)^0.5</f>
         <v>2.1356954354233362</v>
       </c>
+      <c r="AJ69" s="4">
+        <f t="shared" si="11"/>
+        <v>1.0089874689318388E-2</v>
+      </c>
     </row>
-    <row r="70" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="13" t="s">
         <v>15</v>
       </c>
@@ -13350,7 +13413,7 @@
         <v>3253.0000001192093</v>
       </c>
       <c r="AB70" s="15">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="AB70:AB88" si="22">(0.000304*199000000000000000)*EXP(-(5580-680)/(1.987*(C70+273)))</f>
         <v>14820423493.51034</v>
       </c>
       <c r="AC70" s="15">
@@ -13375,8 +13438,12 @@
       </c>
       <c r="AH70" s="37"/>
       <c r="AI70" s="36"/>
+      <c r="AJ70" s="15">
+        <f t="shared" si="11"/>
+        <v>1.0013914627244375E-2</v>
+      </c>
     </row>
-    <row r="71" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>56</v>
       </c>
@@ -13491,8 +13558,12 @@
         <f>(X71^2+AG71^2+AG72^2)^0.5</f>
         <v>2.55747788992654</v>
       </c>
+      <c r="AJ71" s="7">
+        <f t="shared" si="11"/>
+        <v>1.0336612788982173E-2</v>
+      </c>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>15</v>
       </c>
@@ -13608,8 +13679,12 @@
         <f>(X72^2+AG73^2)^0.5</f>
         <v>1.3617023439940106</v>
       </c>
+      <c r="AJ72" s="4">
+        <f t="shared" si="11"/>
+        <v>6.6419721632044858E-3</v>
+      </c>
     </row>
-    <row r="73" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="13" t="s">
         <v>15</v>
       </c>
@@ -13727,8 +13802,12 @@
       </c>
       <c r="AH73" s="37"/>
       <c r="AI73" s="36"/>
+      <c r="AJ73" s="15">
+        <f t="shared" si="11"/>
+        <v>6.5913943964779195E-3</v>
+      </c>
     </row>
-    <row r="74" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>58</v>
       </c>
@@ -13843,8 +13922,12 @@
         <f>(X74^2+AG74^2+AG75^2)^0.5</f>
         <v>1.5986131603737967</v>
       </c>
+      <c r="AJ74" s="7">
+        <f t="shared" ref="AJ74:AJ88" si="31">0.2*AF74/($B$89-Y74)</f>
+        <v>6.7708674761673511E-3</v>
+      </c>
     </row>
-    <row r="75" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>15</v>
       </c>
@@ -13960,8 +14043,12 @@
         <f>(X75^2+AG76^2)^0.5</f>
         <v>0.77871137176683403</v>
       </c>
+      <c r="AJ75" s="4">
+        <f t="shared" si="31"/>
+        <v>3.8816449073328595E-3</v>
+      </c>
     </row>
-    <row r="76" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="13" t="s">
         <v>15</v>
       </c>
@@ -14079,8 +14166,12 @@
       </c>
       <c r="AH76" s="37"/>
       <c r="AI76" s="36"/>
+      <c r="AJ76" s="15">
+        <f t="shared" si="31"/>
+        <v>3.8515088167591573E-3</v>
+      </c>
     </row>
-    <row r="77" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>60</v>
       </c>
@@ -14195,8 +14286,12 @@
         <f>(X77^2+AG77^2+AG78^2)^0.5</f>
         <v>3.2490485062783758</v>
       </c>
+      <c r="AJ77" s="7">
+        <f t="shared" si="31"/>
+        <v>5.1919139706597412E-3</v>
+      </c>
     </row>
-    <row r="78" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>15</v>
       </c>
@@ -14312,8 +14407,12 @@
         <f>(X78^2+AG79^2)^0.5</f>
         <v>1.6885512021665219</v>
       </c>
+      <c r="AJ78" s="4">
+        <f t="shared" si="31"/>
+        <v>1.14522692313179E-2</v>
+      </c>
     </row>
-    <row r="79" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="13" t="s">
         <v>15</v>
       </c>
@@ -14431,8 +14530,12 @@
       </c>
       <c r="AH79" s="37"/>
       <c r="AI79" s="36"/>
+      <c r="AJ79" s="15">
+        <f t="shared" si="31"/>
+        <v>1.1378393820399285E-2</v>
+      </c>
     </row>
-    <row r="80" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>62</v>
       </c>
@@ -14547,8 +14650,12 @@
         <f>(X80^2+AG80^2+AG81^2)^0.5</f>
         <v>1.8876885185255603</v>
       </c>
+      <c r="AJ80" s="7">
+        <f t="shared" si="31"/>
+        <v>1.1949134575028969E-2</v>
+      </c>
     </row>
-    <row r="81" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>15</v>
       </c>
@@ -14664,8 +14771,12 @@
         <f>(X81^2+AG82^2)^0.5</f>
         <v>0.73978213196764342</v>
       </c>
+      <c r="AJ81" s="4">
+        <f t="shared" si="31"/>
+        <v>5.2284450643259187E-3</v>
+      </c>
     </row>
-    <row r="82" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A82" s="13" t="s">
         <v>15</v>
       </c>
@@ -14783,8 +14894,12 @@
       </c>
       <c r="AH82" s="37"/>
       <c r="AI82" s="36"/>
+      <c r="AJ82" s="15">
+        <f t="shared" si="31"/>
+        <v>5.1870825709959389E-3</v>
+      </c>
     </row>
-    <row r="83" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
         <v>63</v>
       </c>
@@ -14899,8 +15014,12 @@
         <f>(X83^2+AG83^2+AG84^2)^0.5</f>
         <v>1.4114442681642989</v>
       </c>
+      <c r="AJ83" s="7">
+        <f t="shared" si="31"/>
+        <v>5.449540309742794E-3</v>
+      </c>
     </row>
-    <row r="84" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>15</v>
       </c>
@@ -15016,8 +15135,12 @@
         <f>(X84^2+AG85^2)^0.5</f>
         <v>1.1336855766702543</v>
       </c>
+      <c r="AJ84" s="4">
+        <f t="shared" si="31"/>
+        <v>8.5043572990653425E-3</v>
+      </c>
     </row>
-    <row r="85" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="13" t="s">
         <v>15</v>
       </c>
@@ -15135,8 +15258,12 @@
       </c>
       <c r="AH85" s="37"/>
       <c r="AI85" s="36"/>
+      <c r="AJ85" s="15">
+        <f t="shared" si="31"/>
+        <v>8.4383070373307417E-3</v>
+      </c>
     </row>
-    <row r="86" spans="1:35" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:36" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>42</v>
       </c>
@@ -15251,8 +15378,12 @@
         <f>(X86^2+AG86^2+AG87^2)^0.5</f>
         <v>1.2259902068947057</v>
       </c>
+      <c r="AJ86" s="7">
+        <f t="shared" si="31"/>
+        <v>8.6577159196502378E-3</v>
+      </c>
     </row>
-    <row r="87" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>15</v>
       </c>
@@ -15368,8 +15499,12 @@
         <f>(X87^2+AG88^2)^0.5</f>
         <v>0.40990824125675746</v>
       </c>
+      <c r="AJ87" s="4">
+        <f t="shared" si="31"/>
+        <v>3.0529742884604842E-3</v>
+      </c>
     </row>
-    <row r="88" spans="1:35" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:36" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A88" s="13" t="s">
         <v>15</v>
       </c>
@@ -15487,8 +15622,12 @@
       </c>
       <c r="AH88" s="37"/>
       <c r="AI88" s="36"/>
+      <c r="AJ88" s="15">
+        <f t="shared" si="31"/>
+        <v>3.0297597548226037E-3</v>
+      </c>
     </row>
-    <row r="89" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>132</v>
       </c>
@@ -15690,8 +15829,8 @@
       <c r="C4" s="24">
         <v>240</v>
       </c>
-      <c r="D4" s="24" cm="1">
-        <f t="array" ref="D4:E4">'[1]Raw Data and Corrections'!AG9:AH9</f>
+      <c r="D4" s="62" cm="1">
+        <f t="array" ref="D4:E4">'Raw Data and Corrections'!AH9:AI9</f>
         <v>4.9585314106207479E-2</v>
       </c>
       <c r="E4" s="26">
@@ -15798,8 +15937,8 @@
       <c r="C5" s="24">
         <v>240</v>
       </c>
-      <c r="D5" s="24" cm="1">
-        <f t="array" ref="D5:E5">'[1]Raw Data and Corrections'!AG13:AH13</f>
+      <c r="D5" s="62" cm="1">
+        <f t="array" ref="D5:E5">'Raw Data and Corrections'!AH13:AI13</f>
         <v>1.1125652685248788E-2</v>
       </c>
       <c r="E5" s="26">
@@ -15906,8 +16045,8 @@
       <c r="C6">
         <v>240</v>
       </c>
-      <c r="D6" cm="1">
-        <f t="array" ref="D6:E6">'[1]Raw Data and Corrections'!AG17:AH17</f>
+      <c r="D6" s="31" cm="1">
+        <f t="array" ref="D6:E6">'Raw Data and Corrections'!AH17:AI17</f>
         <v>1.6418388917769666</v>
       </c>
       <c r="E6" s="17">
@@ -15918,7 +16057,7 @@
         <v>14400</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" si="1"/>
+        <f>D6+G5</f>
         <v>1.7025498585684229</v>
       </c>
       <c r="H6">
@@ -15926,7 +16065,7 @@
         <v>0.23438468069743329</v>
       </c>
       <c r="I6" s="4">
-        <f t="shared" si="3"/>
+        <f>G6/$G$29</f>
         <v>2.7569157429746011E-3</v>
       </c>
       <c r="J6" s="4">
@@ -15934,7 +16073,7 @@
         <v>3.7953591366197281E-4</v>
       </c>
       <c r="L6" s="4">
-        <f t="shared" si="5"/>
+        <f>((I6^2-I5^2)*PI())/(36*F6)</f>
         <v>4.6002272531711332E-11</v>
       </c>
       <c r="M6" s="4">
@@ -16012,8 +16151,8 @@
       <c r="C7">
         <v>60</v>
       </c>
-      <c r="D7" cm="1">
-        <f t="array" ref="D7:E7">'[1]Raw Data and Corrections'!AG21:AH21</f>
+      <c r="D7" s="31" cm="1">
+        <f t="array" ref="D7:E7">'Raw Data and Corrections'!AH21:AI21</f>
         <v>3.6974788092208</v>
       </c>
       <c r="E7" s="17">
@@ -16118,8 +16257,8 @@
       <c r="C8">
         <v>60</v>
       </c>
-      <c r="D8" cm="1">
-        <f t="array" ref="D8:E8">'[1]Raw Data and Corrections'!AG25:AH25</f>
+      <c r="D8" s="31" cm="1">
+        <f t="array" ref="D8:E8">'Raw Data and Corrections'!AH25:AI25</f>
         <v>5.2581583200694721</v>
       </c>
       <c r="E8" s="17">
@@ -16224,8 +16363,8 @@
       <c r="C9">
         <v>60</v>
       </c>
-      <c r="D9" cm="1">
-        <f t="array" ref="D9:E9">'[1]Raw Data and Corrections'!AG28:AH28</f>
+      <c r="D9" s="31" cm="1">
+        <f t="array" ref="D9:E9">'Raw Data and Corrections'!AH28:AI28</f>
         <v>8.9926263591844844</v>
       </c>
       <c r="E9" s="17">
@@ -16330,8 +16469,8 @@
       <c r="C10">
         <v>60</v>
       </c>
-      <c r="D10" cm="1">
-        <f t="array" ref="D10:E10">'[1]Raw Data and Corrections'!AG31:AH31</f>
+      <c r="D10" s="31" cm="1">
+        <f t="array" ref="D10:E10">'Raw Data and Corrections'!AH31:AI31</f>
         <v>9.5082280268323043</v>
       </c>
       <c r="E10" s="17">
@@ -16436,8 +16575,8 @@
       <c r="C11">
         <v>60</v>
       </c>
-      <c r="D11" cm="1">
-        <f t="array" ref="D11:E11">'[1]Raw Data and Corrections'!AG35:AH35</f>
+      <c r="D11" s="31" cm="1">
+        <f t="array" ref="D11:E11">'Raw Data and Corrections'!AH35:AI35</f>
         <v>3.5751128512312391</v>
       </c>
       <c r="E11" s="17">
@@ -16542,8 +16681,8 @@
       <c r="C12">
         <v>80</v>
       </c>
-      <c r="D12" cm="1">
-        <f t="array" ref="D12:E12">'[1]Raw Data and Corrections'!AG38:AH38</f>
+      <c r="D12" s="31" cm="1">
+        <f t="array" ref="D12:E12">'Raw Data and Corrections'!AH38:AI38</f>
         <v>2.5210171532273193</v>
       </c>
       <c r="E12" s="17">
@@ -16648,8 +16787,8 @@
       <c r="C13" s="24">
         <v>100</v>
       </c>
-      <c r="D13" s="24" cm="1">
-        <f t="array" ref="D13:E13">'[1]Raw Data and Corrections'!AG41:AH41</f>
+      <c r="D13" s="62" cm="1">
+        <f t="array" ref="D13:E13">'Raw Data and Corrections'!AH41:AI41</f>
         <v>0.60143930751904229</v>
       </c>
       <c r="E13" s="26">
@@ -16756,8 +16895,8 @@
       <c r="C14">
         <v>60</v>
       </c>
-      <c r="D14" cm="1">
-        <f t="array" ref="D14:E14">'[1]Raw Data and Corrections'!AG44:AH44</f>
+      <c r="D14" s="31" cm="1">
+        <f t="array" ref="D14:E14">'Raw Data and Corrections'!AH44:AI44</f>
         <v>6.6769386443019538</v>
       </c>
       <c r="E14" s="17">
@@ -16862,8 +17001,8 @@
       <c r="C15">
         <v>120</v>
       </c>
-      <c r="D15" cm="1">
-        <f t="array" ref="D15:E15">'[1]Raw Data and Corrections'!AG47:AH47</f>
+      <c r="D15" s="31" cm="1">
+        <f t="array" ref="D15:E15">'Raw Data and Corrections'!AH47:AI47</f>
         <v>11.113966590277643</v>
       </c>
       <c r="E15" s="17">
@@ -16968,8 +17107,8 @@
       <c r="C16">
         <v>180</v>
       </c>
-      <c r="D16" cm="1">
-        <f t="array" ref="D16:E16">'[1]Raw Data and Corrections'!AG50:AH50</f>
+      <c r="D16" s="31" cm="1">
+        <f t="array" ref="D16:E16">'Raw Data and Corrections'!AH50:AI50</f>
         <v>13.792105763034851</v>
       </c>
       <c r="E16" s="17">
@@ -17074,8 +17213,8 @@
       <c r="C17">
         <v>60</v>
       </c>
-      <c r="D17" cm="1">
-        <f t="array" ref="D17:E17">'[1]Raw Data and Corrections'!AG53:AH53</f>
+      <c r="D17" s="31" cm="1">
+        <f t="array" ref="D17:E17">'Raw Data and Corrections'!AH53:AI53</f>
         <v>11.358315176506476</v>
       </c>
       <c r="E17" s="17">
@@ -17180,8 +17319,8 @@
       <c r="C18">
         <v>60</v>
       </c>
-      <c r="D18" cm="1">
-        <f t="array" ref="D18:E18">'[1]Raw Data and Corrections'!AG56:AH56</f>
+      <c r="D18" s="31" cm="1">
+        <f t="array" ref="D18:E18">'Raw Data and Corrections'!AH56:AI56</f>
         <v>14.462752797544418</v>
       </c>
       <c r="E18" s="17">
@@ -17286,8 +17425,8 @@
       <c r="C19">
         <v>60</v>
       </c>
-      <c r="D19" cm="1">
-        <f t="array" ref="D19:E19">'[1]Raw Data and Corrections'!AG59:AH59</f>
+      <c r="D19" s="31" cm="1">
+        <f t="array" ref="D19:E19">'Raw Data and Corrections'!AH59:AI59</f>
         <v>28.330053300207055</v>
       </c>
       <c r="E19" s="17">
@@ -17392,8 +17531,8 @@
       <c r="C20">
         <v>60</v>
       </c>
-      <c r="D20" cm="1">
-        <f t="array" ref="D20:E20">'[1]Raw Data and Corrections'!AG62:AH62</f>
+      <c r="D20" s="31" cm="1">
+        <f t="array" ref="D20:E20">'Raw Data and Corrections'!AH62:AI62</f>
         <v>41.343332028472403</v>
       </c>
       <c r="E20" s="17">
@@ -17498,8 +17637,8 @@
       <c r="C21">
         <v>60</v>
       </c>
-      <c r="D21" cm="1">
-        <f t="array" ref="D21:E21">'[1]Raw Data and Corrections'!AG65:AH65</f>
+      <c r="D21" s="31" cm="1">
+        <f t="array" ref="D21:E21">'Raw Data and Corrections'!AH65:AI65</f>
         <v>44.783772075614529</v>
       </c>
       <c r="E21" s="17">
@@ -17606,8 +17745,8 @@
       <c r="C22">
         <v>60</v>
       </c>
-      <c r="D22" cm="1">
-        <f t="array" ref="D22:E22">'[1]Raw Data and Corrections'!AG68:AH68</f>
+      <c r="D22" s="31" cm="1">
+        <f t="array" ref="D22:E22">'Raw Data and Corrections'!AH68:AI68</f>
         <v>15.32951848324867</v>
       </c>
       <c r="E22" s="17">
@@ -17712,8 +17851,8 @@
       <c r="C23">
         <v>60</v>
       </c>
-      <c r="D23" cm="1">
-        <f t="array" ref="D23:E23">'[1]Raw Data and Corrections'!AG71:AH71</f>
+      <c r="D23" s="31" cm="1">
+        <f t="array" ref="D23:E23">'Raw Data and Corrections'!AH71:AI71</f>
         <v>7.4056558378177257</v>
       </c>
       <c r="E23" s="17">
@@ -17818,8 +17957,8 @@
       <c r="C24">
         <v>100</v>
       </c>
-      <c r="D24" cm="1">
-        <f t="array" ref="D24:E24">'[1]Raw Data and Corrections'!AG74:AH74</f>
+      <c r="D24" s="31" cm="1">
+        <f t="array" ref="D24:E24">'Raw Data and Corrections'!AH74:AI74</f>
         <v>6.7885433898562955</v>
       </c>
       <c r="E24" s="17">
@@ -17924,8 +18063,8 @@
       <c r="C25">
         <v>240</v>
       </c>
-      <c r="D25" cm="1">
-        <f t="array" ref="D25:E25">'[1]Raw Data and Corrections'!AG77:AH77</f>
+      <c r="D25" s="31" cm="1">
+        <f t="array" ref="D25:E25">'Raw Data and Corrections'!AH77:AI77</f>
         <v>109.98923129912342</v>
       </c>
       <c r="E25" s="17">
@@ -18030,8 +18169,8 @@
       <c r="C26">
         <v>90</v>
       </c>
-      <c r="D26" cm="1">
-        <f t="array" ref="D26:E26">'[1]Raw Data and Corrections'!AG80:AH80</f>
+      <c r="D26" s="31" cm="1">
+        <f t="array" ref="D26:E26">'Raw Data and Corrections'!AH80:AI80</f>
         <v>5.8007597520409249</v>
       </c>
       <c r="E26" s="17">
@@ -18136,8 +18275,8 @@
       <c r="C27">
         <v>60</v>
       </c>
-      <c r="D27" cm="1">
-        <f t="array" ref="D27:E27">'[1]Raw Data and Corrections'!AG83:AH83</f>
+      <c r="D27" s="31" cm="1">
+        <f t="array" ref="D27:E27">'Raw Data and Corrections'!AH83:AI83</f>
         <v>18.117517289967918</v>
       </c>
       <c r="E27" s="17">
@@ -18242,8 +18381,8 @@
       <c r="C28" s="24">
         <v>120</v>
       </c>
-      <c r="D28" s="24" cm="1">
-        <f t="array" ref="D28:E28">'[1]Raw Data and Corrections'!AG86:AH86</f>
+      <c r="D28" s="62" cm="1">
+        <f t="array" ref="D28:E28">'Raw Data and Corrections'!AH86:AI86</f>
         <v>0.70246648635252917</v>
       </c>
       <c r="E28" s="26">

</xml_diff>